<commit_message>
new data new day new model new vibes
</commit_message>
<xml_diff>
--- a/data/treatment_key.xlsx
+++ b/data/treatment_key.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/graceleuchtenberger/Library/Mobile Documents/com~apple~CloudDocs/Documents/Density_field/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CCFD09B7-5BD2-D64B-A8A1-A7BC719ABB3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AED08280-AE76-864A-B2CD-CA887EC1F6B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13500" yWindow="2480" windowWidth="28040" windowHeight="17440" xr2:uid="{D9A139D6-922D-CE47-B760-C8C11F9B1470}"/>
+    <workbookView xWindow="10080" yWindow="540" windowWidth="28040" windowHeight="17440" xr2:uid="{D9A139D6-922D-CE47-B760-C8C11F9B1470}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="30">
   <si>
     <t>bag_num</t>
   </si>
@@ -53,9 +53,6 @@
     <t>S</t>
   </si>
   <si>
-    <t>C</t>
-  </si>
-  <si>
     <t>H</t>
   </si>
   <si>
@@ -72,6 +69,63 @@
   </si>
   <si>
     <t>rack</t>
+  </si>
+  <si>
+    <t>93-2</t>
+  </si>
+  <si>
+    <t>95-1</t>
+  </si>
+  <si>
+    <t>45-2</t>
+  </si>
+  <si>
+    <t>45-1</t>
+  </si>
+  <si>
+    <t>43-2</t>
+  </si>
+  <si>
+    <t>44-1</t>
+  </si>
+  <si>
+    <t>93-1</t>
+  </si>
+  <si>
+    <t>94-1</t>
+  </si>
+  <si>
+    <t>95-2</t>
+  </si>
+  <si>
+    <t>97-1</t>
+  </si>
+  <si>
+    <t>29-1</t>
+  </si>
+  <si>
+    <t>27-1</t>
+  </si>
+  <si>
+    <t>28-2</t>
+  </si>
+  <si>
+    <t>28-1</t>
+  </si>
+  <si>
+    <t>43-1</t>
+  </si>
+  <si>
+    <t>98-1</t>
+  </si>
+  <si>
+    <t>98-2</t>
+  </si>
+  <si>
+    <t>99-1</t>
+  </si>
+  <si>
+    <t>top_bottom</t>
   </si>
 </sst>
 </file>
@@ -443,10 +497,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5150AFA3-C786-F14A-A9B2-6B43899C6D2C}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -457,49 +511,58 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
         <v>8</v>
       </c>
-      <c r="E1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>93</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
       <c r="E2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>94</v>
+      <c r="F2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>95</v>
+      <c r="F3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>13</v>
       </c>
       <c r="B4" t="s">
         <v>1</v>
@@ -513,13 +576,16 @@
       <c r="E4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>96</v>
+      <c r="F4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C5" t="s">
         <v>6</v>
@@ -530,101 +596,119 @@
       <c r="E5" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>97</v>
+      <c r="F5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C6" t="s">
         <v>6</v>
       </c>
       <c r="D6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>98</v>
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C7" t="s">
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E7" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>99</v>
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D8" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>100</v>
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>18</v>
       </c>
       <c r="B9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" t="s">
         <v>5</v>
       </c>
-      <c r="C9" t="s">
-        <v>6</v>
-      </c>
       <c r="D9" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E9" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>27</v>
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E10" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>28</v>
+        <v>1</v>
+      </c>
+      <c r="F10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D11" t="s">
         <v>9</v>
@@ -632,107 +716,168 @@
       <c r="E11" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>29</v>
+      <c r="F11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>21</v>
       </c>
       <c r="B12" t="s">
         <v>4</v>
       </c>
       <c r="C12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" t="s">
+        <v>4</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" t="s">
+        <v>4</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" t="s">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>6</v>
+      </c>
+      <c r="D14" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" t="s">
+        <v>4</v>
+      </c>
+      <c r="F14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>6</v>
+      </c>
+      <c r="D15" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" t="s">
+        <v>4</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" t="s">
         <v>9</v>
       </c>
-      <c r="E12" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>30</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="E16" t="s">
+        <v>1</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
         <v>5</v>
       </c>
-      <c r="C13" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" t="s">
+      <c r="D17" t="s">
         <v>9</v>
       </c>
-      <c r="E13" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14">
-        <v>43</v>
-      </c>
-      <c r="B14" t="s">
-        <v>1</v>
-      </c>
-      <c r="C14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E14" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15">
-        <v>44</v>
-      </c>
-      <c r="B15" t="s">
-        <v>4</v>
-      </c>
-      <c r="C15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" t="s">
-        <v>10</v>
-      </c>
-      <c r="E15" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16">
-        <v>45</v>
-      </c>
-      <c r="B16" t="s">
-        <v>1</v>
-      </c>
-      <c r="C16" t="s">
-        <v>7</v>
-      </c>
-      <c r="D16" t="s">
-        <v>10</v>
-      </c>
-      <c r="E16" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17">
-        <v>46</v>
-      </c>
-      <c r="B17" t="s">
+      <c r="E17" t="s">
+        <v>4</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" t="s">
         <v>5</v>
       </c>
-      <c r="C17" t="s">
-        <v>7</v>
-      </c>
-      <c r="D17" t="s">
-        <v>10</v>
-      </c>
-      <c r="E17" t="s">
-        <v>1</v>
+      <c r="D18" t="s">
+        <v>9</v>
+      </c>
+      <c r="E18" t="s">
+        <v>4</v>
+      </c>
+      <c r="F18">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" t="s">
+        <v>5</v>
+      </c>
+      <c r="D19" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19" t="s">
+        <v>4</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>